<commit_message>
Add the Spanish solar-anchored import scenarios to scenarios_clean
Two new rows: iron made in Spain from an islanded, solar-anchored RES mix
at the p95 best site, melted to steel in Germany and in France
(import-ESP-GER- and import-ESP-FRA-h2-dri-eaf-res-mix-solar-p95). The
other 398 scenarios and the assumptions_inputs tab are unchanged.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/assumptions/Assumptions_yaml_inputs.xlsx
+++ b/data/assumptions/Assumptions_yaml_inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hannah.maral\Documents\LCOX\lcox-steel\data\assumptions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54DC8B21-E511-4A52-8360-6E2F8581487C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A0FDC87-9713-4242-9C38-B51E42CE15BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="86280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{92D1E11C-B21A-48C9-8540-2467AF5A4842}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{92D1E11C-B21A-48C9-8540-2467AF5A4842}"/>
   </bookViews>
   <sheets>
     <sheet name="assumptions_inputs" sheetId="6" r:id="rId1"/>
@@ -138,7 +138,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5065" uniqueCount="615">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5089" uniqueCount="617">
   <si>
     <t>YAML key</t>
   </si>
@@ -1983,6 +1983,12 @@
   </si>
   <si>
     <t>shipping.cost_eur_per_t</t>
+  </si>
+  <si>
+    <t>import-ESP-GER-h2-dri-eaf-res-mix-solar-p95</t>
+  </si>
+  <si>
+    <t>import-ESP-FRA-h2-dri-eaf-res-mix-solar-p95</t>
   </si>
 </sst>
 </file>
@@ -2131,7 +2137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -2187,6 +2193,7 @@
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2703,7 +2710,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="6">
+  <wetp:taskpane dockstate="right" visibility="0" width="554" row="6">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -4603,7 +4610,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03D668BA-3BF5-48C5-8A75-05846F0671CD}">
-  <dimension ref="A1:M399"/>
+  <dimension ref="A1:M401"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.45">
@@ -19696,78 +19703,156 @@
       </c>
     </row>
     <row r="398" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="A398" t="s">
+      <c r="A398" s="19" t="s">
+        <v>615</v>
+      </c>
+      <c r="B398" s="19" t="s">
+        <v>297</v>
+      </c>
+      <c r="C398" s="19" t="s">
+        <v>149</v>
+      </c>
+      <c r="D398" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="E398" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="F398" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="G398" s="19" t="s">
+        <v>100</v>
+      </c>
+      <c r="H398" s="19"/>
+      <c r="I398" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="J398" s="19" t="s">
+        <v>102</v>
+      </c>
+      <c r="K398" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="L398" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="M398" s="19" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="399" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A399" s="19" t="s">
+        <v>616</v>
+      </c>
+      <c r="B399" s="19" t="s">
+        <v>297</v>
+      </c>
+      <c r="C399" s="19" t="s">
+        <v>149</v>
+      </c>
+      <c r="D399" s="19" t="s">
+        <v>186</v>
+      </c>
+      <c r="E399" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="F399" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="G399" s="19" t="s">
+        <v>100</v>
+      </c>
+      <c r="H399" s="19"/>
+      <c r="I399" s="19" t="s">
+        <v>101</v>
+      </c>
+      <c r="J399" s="19" t="s">
+        <v>102</v>
+      </c>
+      <c r="K399" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="L399" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="M399" s="19" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="400" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A400" t="s">
         <v>513</v>
       </c>
-      <c r="B398" t="s">
+      <c r="B400" t="s">
         <v>96</v>
       </c>
-      <c r="C398" t="s">
+      <c r="C400" t="s">
         <v>97</v>
       </c>
-      <c r="D398" t="s">
+      <c r="D400" t="s">
         <v>97</v>
       </c>
-      <c r="E398" t="s">
+      <c r="E400" t="s">
         <v>98</v>
       </c>
-      <c r="F398" t="s">
-        <v>99</v>
-      </c>
-      <c r="G398" t="s">
+      <c r="F400" t="s">
+        <v>99</v>
+      </c>
+      <c r="G400" t="s">
         <v>100</v>
       </c>
-      <c r="I398" t="s">
+      <c r="I400" t="s">
         <v>107</v>
       </c>
-      <c r="J398" t="s">
-        <v>102</v>
-      </c>
-      <c r="K398" t="s">
-        <v>103</v>
-      </c>
-      <c r="L398" t="s">
-        <v>104</v>
-      </c>
-      <c r="M398" t="s">
+      <c r="J400" t="s">
+        <v>102</v>
+      </c>
+      <c r="K400" t="s">
+        <v>103</v>
+      </c>
+      <c r="L400" t="s">
+        <v>104</v>
+      </c>
+      <c r="M400" t="s">
         <v>514</v>
       </c>
     </row>
-    <row r="399" spans="1:13" x14ac:dyDescent="0.45">
-      <c r="A399" t="s">
+    <row r="401" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A401" t="s">
         <v>515</v>
       </c>
-      <c r="B399" t="s">
+      <c r="B401" t="s">
         <v>96</v>
       </c>
-      <c r="C399" t="s">
+      <c r="C401" t="s">
         <v>97</v>
       </c>
-      <c r="D399" t="s">
+      <c r="D401" t="s">
         <v>97</v>
       </c>
-      <c r="E399" t="s">
+      <c r="E401" t="s">
         <v>98</v>
       </c>
-      <c r="F399" t="s">
-        <v>99</v>
-      </c>
-      <c r="G399" t="s">
+      <c r="F401" t="s">
+        <v>99</v>
+      </c>
+      <c r="G401" t="s">
         <v>100</v>
       </c>
-      <c r="I399" t="s">
+      <c r="I401" t="s">
         <v>107</v>
       </c>
-      <c r="J399" t="s">
-        <v>102</v>
-      </c>
-      <c r="K399" t="s">
-        <v>103</v>
-      </c>
-      <c r="L399" t="s">
-        <v>104</v>
-      </c>
-      <c r="M399" t="s">
+      <c r="J401" t="s">
+        <v>102</v>
+      </c>
+      <c r="K401" t="s">
+        <v>103</v>
+      </c>
+      <c r="L401" t="s">
+        <v>104</v>
+      </c>
+      <c r="M401" t="s">
         <v>516</v>
       </c>
     </row>

</xml_diff>